<commit_message>
Update RSS CSV & Excel (reporting)
</commit_message>
<xml_diff>
--- a/output/rss_history.xlsx
+++ b/output/rss_history.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E402"/>
+  <dimension ref="A1:E403"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -11183,6 +11183,29 @@
       <c r="E402" t="inlineStr">
         <is>
           <t>5. Logiciels _ OS</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>Frandroid - Actualités</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr"/>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>Comment bien choisir son clavier ?</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>https://native.humanoid.fr/register-click?s_id=2&amp;sp_id=47&amp;c_id=4226</t>
+        </is>
+      </c>
+      <c r="E403" t="inlineStr">
+        <is>
+          <t>3. Periphérique</t>
         </is>
       </c>
     </row>
@@ -20257,7 +20280,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20606,6 +20629,29 @@
         </is>
       </c>
       <c r="E13" t="inlineStr">
+        <is>
+          <t>3. Periphérique</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Frandroid - Actualités</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Comment bien choisir son clavier ?</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://native.humanoid.fr/register-click?s_id=2&amp;sp_id=47&amp;c_id=4226</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>3. Periphérique</t>
         </is>

</xml_diff>